<commit_message>
Fix EAM category import ordering and preview response handling
</commit_message>
<xml_diff>
--- a/backend/yudao-module-eam/src/main/resources/eam/eam-category-config-template.xlsx
+++ b/backend/yudao-module-eam/src/main/resources/eam/eam-category-config-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类" sheetId="1" r:id="R52fe59ab6bbb4773"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段" sheetId="2" r:id="R24c61725997541dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分类" sheetId="1" r:id="R93a8d41c06dd497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段" sheetId="2" r:id="Rb1a586a4b4584478"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -577,7 +577,7 @@
       <x:c r="B2" s="9" t="str">
         <x:v>IT硬件设备</x:v>
       </x:c>
-      <x:c r="C2" s="9" t="str"/>
+      <x:c r="C2" s="9"/>
       <x:c r="D2" s="9" t="str">
         <x:v>开启</x:v>
       </x:c>
@@ -602,25 +602,23 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="22" t="str">
-        <x:v>IT-COMPUTER</x:v>
+        <x:v>DIGITAL</x:v>
       </x:c>
       <x:c r="B3" s="12" t="str">
-        <x:v>电脑</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="str">
-        <x:v>IT</x:v>
-      </x:c>
+        <x:v>数字资产</x:v>
+      </x:c>
+      <x:c r="C3" s="12"/>
       <x:c r="D3" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E3" s="12" t="str">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F3" s="12" t="str">
         <x:v>单件</x:v>
       </x:c>
       <x:c r="G3" s="12" t="str">
-        <x:v>台</x:v>
+        <x:v>项</x:v>
       </x:c>
       <x:c r="H3" s="12" t="str">
         <x:v>V3</x:v>
@@ -634,25 +632,23 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="22" t="str">
-        <x:v>DIGITAL-PLATFORM</x:v>
+        <x:v>FURNITURE</x:v>
       </x:c>
       <x:c r="B4" s="12" t="str">
-        <x:v>平台账号</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="str">
-        <x:v>DIGITAL</x:v>
-      </x:c>
+        <x:v>办公家具及设备</x:v>
+      </x:c>
+      <x:c r="C4" s="12"/>
       <x:c r="D4" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F4" s="12" t="str">
         <x:v>单件</x:v>
       </x:c>
       <x:c r="G4" s="12" t="str">
-        <x:v>个</x:v>
+        <x:v>件</x:v>
       </x:c>
       <x:c r="H4" s="12" t="str">
         <x:v>V3</x:v>
@@ -666,25 +662,23 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="22" t="str">
-        <x:v>FURNITURE-DESK-CHAIR</x:v>
+        <x:v>SUPPLIES</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>办公桌椅</x:v>
-      </x:c>
-      <x:c r="C5" s="12" t="str">
-        <x:v>FURNITURE</x:v>
-      </x:c>
+        <x:v>办公用品和耗材</x:v>
+      </x:c>
+      <x:c r="C5" s="12"/>
       <x:c r="D5" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>单件</x:v>
+        <x:v>批量</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
-        <x:v>件</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
         <x:v>V3</x:v>
@@ -698,25 +692,23 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="22" t="str">
-        <x:v>SUPPLIES-STATIONERY</x:v>
+        <x:v>BOOK</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>文具</x:v>
-      </x:c>
-      <x:c r="C6" s="12" t="str">
-        <x:v>SUPPLIES</x:v>
-      </x:c>
+        <x:v>专业书籍</x:v>
+      </x:c>
+      <x:c r="C6" s="12"/>
       <x:c r="D6" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
         <x:v>批量</x:v>
       </x:c>
       <x:c r="G6" s="12" t="str">
-        <x:v>个</x:v>
+        <x:v>册</x:v>
       </x:c>
       <x:c r="H6" s="12" t="str">
         <x:v>V3</x:v>
@@ -730,19 +722,17 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="22" t="str">
-        <x:v>TEACHING-KITCHEN-SCALE</x:v>
+        <x:v>TEACHING</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>厨房秤</x:v>
-      </x:c>
-      <x:c r="C7" s="12" t="str">
-        <x:v>TEACHING</x:v>
-      </x:c>
+        <x:v>教学用具</x:v>
+      </x:c>
+      <x:c r="C7" s="12"/>
       <x:c r="D7" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
         <x:v>批量</x:v>
@@ -762,19 +752,17 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="22" t="str">
-        <x:v>OTHER-ASSET</x:v>
+        <x:v>OTHER</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>其他资产</x:v>
-      </x:c>
-      <x:c r="C8" s="12" t="str">
-        <x:v>OTHER</x:v>
-      </x:c>
+        <x:v>其他</x:v>
+      </x:c>
+      <x:c r="C8" s="12"/>
       <x:c r="D8" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>1</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
         <x:v>单件</x:v>
@@ -794,23 +782,25 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="22" t="str">
-        <x:v>DIGITAL</x:v>
+        <x:v>IT-COMPUTER</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>数字资产</x:v>
-      </x:c>
-      <x:c r="C9" s="12" t="str"/>
+        <x:v>电脑</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="str">
+        <x:v>IT</x:v>
+      </x:c>
       <x:c r="D9" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
         <x:v>单件</x:v>
       </x:c>
       <x:c r="G9" s="12" t="str">
-        <x:v>项</x:v>
+        <x:v>台</x:v>
       </x:c>
       <x:c r="H9" s="12" t="str">
         <x:v>V3</x:v>
@@ -824,25 +814,25 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="22" t="str">
-        <x:v>IT-MOBILE</x:v>
+        <x:v>DIGITAL-PLATFORM</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>移动终端</x:v>
+        <x:v>平台账号</x:v>
       </x:c>
       <x:c r="C10" s="12" t="str">
-        <x:v>IT</x:v>
+        <x:v>DIGITAL</x:v>
       </x:c>
       <x:c r="D10" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E10" s="12" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
         <x:v>单件</x:v>
       </x:c>
       <x:c r="G10" s="12" t="str">
-        <x:v>台</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="H10" s="12" t="str">
         <x:v>V3</x:v>
@@ -856,25 +846,25 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="22" t="str">
-        <x:v>DIGITAL-SUBSCRIPTION</x:v>
+        <x:v>FURNITURE-DESK-CHAIR</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>订阅服务</x:v>
+        <x:v>办公桌椅</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>DIGITAL</x:v>
+        <x:v>FURNITURE</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
         <x:v>单件</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
-        <x:v>项</x:v>
+        <x:v>件</x:v>
       </x:c>
       <x:c r="H11" s="12" t="str">
         <x:v>V3</x:v>
@@ -888,25 +878,25 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="22" t="str">
-        <x:v>FURNITURE-RECEPTION</x:v>
+        <x:v>SUPPLIES-STATIONERY</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>会客家具</x:v>
+        <x:v>文具</x:v>
       </x:c>
       <x:c r="C12" s="12" t="str">
-        <x:v>FURNITURE</x:v>
+        <x:v>SUPPLIES</x:v>
       </x:c>
       <x:c r="D12" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E12" s="12" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>单件</x:v>
+        <x:v>批量</x:v>
       </x:c>
       <x:c r="G12" s="12" t="str">
-        <x:v>件</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
         <x:v>V3</x:v>
@@ -920,25 +910,25 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="22" t="str">
-        <x:v>SUPPLIES-ADHESIVE</x:v>
+        <x:v>TEACHING-KITCHEN-SCALE</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
-        <x:v>胶粘用品</x:v>
+        <x:v>厨房秤</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>SUPPLIES</x:v>
+        <x:v>TEACHING</x:v>
       </x:c>
       <x:c r="D13" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E13" s="12" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F13" s="12" t="str">
         <x:v>批量</x:v>
       </x:c>
       <x:c r="G13" s="12" t="str">
-        <x:v>个</x:v>
+        <x:v>件</x:v>
       </x:c>
       <x:c r="H13" s="12" t="str">
         <x:v>V3</x:v>
@@ -952,25 +942,25 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="22" t="str">
-        <x:v>TEACHING-SANDBOX</x:v>
+        <x:v>OTHER-ASSET</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>沙盘</x:v>
+        <x:v>其他资产</x:v>
       </x:c>
       <x:c r="C14" s="12" t="str">
-        <x:v>TEACHING</x:v>
+        <x:v>OTHER</x:v>
       </x:c>
       <x:c r="D14" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E14" s="12" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>批量</x:v>
+        <x:v>单件</x:v>
       </x:c>
       <x:c r="G14" s="12" t="str">
-        <x:v>件</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="H14" s="12" t="str">
         <x:v>V3</x:v>
@@ -984,23 +974,25 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="22" t="str">
-        <x:v>FURNITURE</x:v>
+        <x:v>IT-MOBILE</x:v>
       </x:c>
       <x:c r="B15" s="12" t="str">
-        <x:v>办公家具及设备</x:v>
-      </x:c>
-      <x:c r="C15" s="12" t="str"/>
+        <x:v>移动终端</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="str">
+        <x:v>IT</x:v>
+      </x:c>
       <x:c r="D15" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E15" s="12" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F15" s="12" t="str">
         <x:v>单件</x:v>
       </x:c>
       <x:c r="G15" s="12" t="str">
-        <x:v>件</x:v>
+        <x:v>台</x:v>
       </x:c>
       <x:c r="H15" s="12" t="str">
         <x:v>V3</x:v>
@@ -1014,25 +1006,25 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="22" t="str">
-        <x:v>IT-DISPLAY</x:v>
+        <x:v>DIGITAL-SUBSCRIPTION</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>显示器</x:v>
+        <x:v>订阅服务</x:v>
       </x:c>
       <x:c r="C16" s="12" t="str">
-        <x:v>IT</x:v>
+        <x:v>DIGITAL</x:v>
       </x:c>
       <x:c r="D16" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E16" s="12" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
         <x:v>单件</x:v>
       </x:c>
       <x:c r="G16" s="12" t="str">
-        <x:v>台</x:v>
+        <x:v>项</x:v>
       </x:c>
       <x:c r="H16" s="12" t="str">
         <x:v>V3</x:v>
@@ -1046,25 +1038,25 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="22" t="str">
-        <x:v>DIGITAL-MOBILE</x:v>
+        <x:v>FURNITURE-RECEPTION</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
-        <x:v>企业手机号</x:v>
+        <x:v>会客家具</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
-        <x:v>DIGITAL</x:v>
+        <x:v>FURNITURE</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E17" s="12" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F17" s="12" t="str">
         <x:v>单件</x:v>
       </x:c>
       <x:c r="G17" s="12" t="str">
-        <x:v>个</x:v>
+        <x:v>件</x:v>
       </x:c>
       <x:c r="H17" s="12" t="str">
         <x:v>V3</x:v>
@@ -1078,25 +1070,25 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="22" t="str">
-        <x:v>FURNITURE-CABINET</x:v>
+        <x:v>SUPPLIES-ADHESIVE</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
-        <x:v>文件柜</x:v>
+        <x:v>胶粘用品</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>FURNITURE</x:v>
+        <x:v>SUPPLIES</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
-        <x:v>单件</x:v>
+        <x:v>批量</x:v>
       </x:c>
       <x:c r="G18" s="12" t="str">
-        <x:v>件</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="H18" s="12" t="str">
         <x:v>V3</x:v>
@@ -1110,25 +1102,25 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="22" t="str">
-        <x:v>SUPPLIES-BATTERY</x:v>
+        <x:v>TEACHING-SANDBOX</x:v>
       </x:c>
       <x:c r="B19" s="12" t="str">
-        <x:v>电池</x:v>
+        <x:v>沙盘</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>SUPPLIES</x:v>
+        <x:v>TEACHING</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E19" s="12" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F19" s="12" t="str">
         <x:v>批量</x:v>
       </x:c>
       <x:c r="G19" s="12" t="str">
-        <x:v>个</x:v>
+        <x:v>件</x:v>
       </x:c>
       <x:c r="H19" s="12" t="str">
         <x:v>V3</x:v>
@@ -1142,13 +1134,13 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="22" t="str">
-        <x:v>TEACHING-PAGODA</x:v>
+        <x:v>IT-DISPLAY</x:v>
       </x:c>
       <x:c r="B20" s="12" t="str">
-        <x:v>膳食宝塔</x:v>
+        <x:v>显示器</x:v>
       </x:c>
       <x:c r="C20" s="12" t="str">
-        <x:v>TEACHING</x:v>
+        <x:v>IT</x:v>
       </x:c>
       <x:c r="D20" s="12" t="str">
         <x:v>开启</x:v>
@@ -1157,10 +1149,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F20" s="12" t="str">
-        <x:v>批量</x:v>
+        <x:v>单件</x:v>
       </x:c>
       <x:c r="G20" s="12" t="str">
-        <x:v>件</x:v>
+        <x:v>台</x:v>
       </x:c>
       <x:c r="H20" s="12" t="str">
         <x:v>V3</x:v>
@@ -1174,20 +1166,22 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="22" t="str">
-        <x:v>SUPPLIES</x:v>
+        <x:v>DIGITAL-MOBILE</x:v>
       </x:c>
       <x:c r="B21" s="12" t="str">
-        <x:v>办公用品和耗材</x:v>
-      </x:c>
-      <x:c r="C21" s="12" t="str"/>
+        <x:v>企业手机号</x:v>
+      </x:c>
+      <x:c r="C21" s="12" t="str">
+        <x:v>DIGITAL</x:v>
+      </x:c>
       <x:c r="D21" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E21" s="12" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F21" s="12" t="str">
-        <x:v>批量</x:v>
+        <x:v>单件</x:v>
       </x:c>
       <x:c r="G21" s="12" t="str">
         <x:v>个</x:v>
@@ -1204,25 +1198,25 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="22" t="str">
-        <x:v>IT-PRINT-PROJECT</x:v>
+        <x:v>FURNITURE-CABINET</x:v>
       </x:c>
       <x:c r="B22" s="12" t="str">
-        <x:v>打印/投影设备</x:v>
+        <x:v>文件柜</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
-        <x:v>IT</x:v>
+        <x:v>FURNITURE</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
         <x:v>单件</x:v>
       </x:c>
       <x:c r="G22" s="12" t="str">
-        <x:v>台</x:v>
+        <x:v>件</x:v>
       </x:c>
       <x:c r="H22" s="12" t="str">
         <x:v>V3</x:v>
@@ -1236,25 +1230,25 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="22" t="str">
-        <x:v>DIGITAL-OTHER</x:v>
+        <x:v>SUPPLIES-BATTERY</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
-        <x:v>其他数字资产</x:v>
+        <x:v>电池</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
-        <x:v>DIGITAL</x:v>
+        <x:v>SUPPLIES</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E23" s="12" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F23" s="12" t="str">
-        <x:v>单件</x:v>
+        <x:v>批量</x:v>
       </x:c>
       <x:c r="G23" s="12" t="str">
-        <x:v>项</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="H23" s="12" t="str">
         <x:v>V3</x:v>
@@ -1268,25 +1262,25 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="22" t="str">
-        <x:v>FURNITURE-WATER</x:v>
+        <x:v>TEACHING-PAGODA</x:v>
       </x:c>
       <x:c r="B24" s="12" t="str">
-        <x:v>饮水机</x:v>
+        <x:v>膳食宝塔</x:v>
       </x:c>
       <x:c r="C24" s="12" t="str">
-        <x:v>FURNITURE</x:v>
+        <x:v>TEACHING</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E24" s="12" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F24" s="12" t="str">
-        <x:v>单件</x:v>
+        <x:v>批量</x:v>
       </x:c>
       <x:c r="G24" s="12" t="str">
-        <x:v>台</x:v>
+        <x:v>件</x:v>
       </x:c>
       <x:c r="H24" s="12" t="str">
         <x:v>V3</x:v>
@@ -1300,13 +1294,13 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="22" t="str">
-        <x:v>SUPPLIES-ARCHIVE</x:v>
+        <x:v>IT-PRINT-PROJECT</x:v>
       </x:c>
       <x:c r="B25" s="12" t="str">
-        <x:v>档案及证书物料</x:v>
+        <x:v>打印/投影设备</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>SUPPLIES</x:v>
+        <x:v>IT</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
         <x:v>开启</x:v>
@@ -1315,10 +1309,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F25" s="12" t="str">
-        <x:v>批量</x:v>
+        <x:v>单件</x:v>
       </x:c>
       <x:c r="G25" s="12" t="str">
-        <x:v>个</x:v>
+        <x:v>台</x:v>
       </x:c>
       <x:c r="H25" s="12" t="str">
         <x:v>V3</x:v>
@@ -1332,13 +1326,13 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="22" t="str">
-        <x:v>TEACHING-PLATE</x:v>
+        <x:v>DIGITAL-OTHER</x:v>
       </x:c>
       <x:c r="B26" s="12" t="str">
-        <x:v>膳食餐盘</x:v>
+        <x:v>其他数字资产</x:v>
       </x:c>
       <x:c r="C26" s="12" t="str">
-        <x:v>TEACHING</x:v>
+        <x:v>DIGITAL</x:v>
       </x:c>
       <x:c r="D26" s="12" t="str">
         <x:v>开启</x:v>
@@ -1347,10 +1341,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F26" s="12" t="str">
-        <x:v>批量</x:v>
+        <x:v>单件</x:v>
       </x:c>
       <x:c r="G26" s="12" t="str">
-        <x:v>件</x:v>
+        <x:v>项</x:v>
       </x:c>
       <x:c r="H26" s="12" t="str">
         <x:v>V3</x:v>
@@ -1364,23 +1358,25 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="22" t="str">
-        <x:v>BOOK</x:v>
+        <x:v>FURNITURE-WATER</x:v>
       </x:c>
       <x:c r="B27" s="12" t="str">
-        <x:v>专业书籍</x:v>
-      </x:c>
-      <x:c r="C27" s="12" t="str"/>
+        <x:v>饮水机</x:v>
+      </x:c>
+      <x:c r="C27" s="12" t="str">
+        <x:v>FURNITURE</x:v>
+      </x:c>
       <x:c r="D27" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E27" s="12" t="str">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F27" s="12" t="str">
-        <x:v>批量</x:v>
+        <x:v>单件</x:v>
       </x:c>
       <x:c r="G27" s="12" t="str">
-        <x:v>册</x:v>
+        <x:v>台</x:v>
       </x:c>
       <x:c r="H27" s="12" t="str">
         <x:v>V3</x:v>
@@ -1394,25 +1390,25 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="22" t="str">
-        <x:v>IT-NETWORK</x:v>
+        <x:v>SUPPLIES-ARCHIVE</x:v>
       </x:c>
       <x:c r="B28" s="12" t="str">
-        <x:v>网络及通讯设备</x:v>
+        <x:v>档案及证书物料</x:v>
       </x:c>
       <x:c r="C28" s="12" t="str">
-        <x:v>IT</x:v>
+        <x:v>SUPPLIES</x:v>
       </x:c>
       <x:c r="D28" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E28" s="12" t="str">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F28" s="12" t="str">
-        <x:v>单件</x:v>
+        <x:v>批量</x:v>
       </x:c>
       <x:c r="G28" s="12" t="str">
-        <x:v>台</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="H28" s="12" t="str">
         <x:v>V3</x:v>
@@ -1426,22 +1422,22 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="22" t="str">
-        <x:v>FURNITURE-OTHER</x:v>
+        <x:v>TEACHING-PLATE</x:v>
       </x:c>
       <x:c r="B29" s="12" t="str">
-        <x:v>其他办公家具及设备</x:v>
+        <x:v>膳食餐盘</x:v>
       </x:c>
       <x:c r="C29" s="12" t="str">
-        <x:v>FURNITURE</x:v>
+        <x:v>TEACHING</x:v>
       </x:c>
       <x:c r="D29" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E29" s="12" t="str">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F29" s="12" t="str">
-        <x:v>单件</x:v>
+        <x:v>批量</x:v>
       </x:c>
       <x:c r="G29" s="12" t="str">
         <x:v>件</x:v>
@@ -1458,13 +1454,13 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="22" t="str">
-        <x:v>SUPPLIES-PRINT</x:v>
+        <x:v>IT-NETWORK</x:v>
       </x:c>
       <x:c r="B30" s="12" t="str">
-        <x:v>印刷物料</x:v>
+        <x:v>网络及通讯设备</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>SUPPLIES</x:v>
+        <x:v>IT</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
         <x:v>开启</x:v>
@@ -1473,10 +1469,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
-        <x:v>批量</x:v>
+        <x:v>单件</x:v>
       </x:c>
       <x:c r="G30" s="12" t="str">
-        <x:v>个</x:v>
+        <x:v>台</x:v>
       </x:c>
       <x:c r="H30" s="12" t="str">
         <x:v>V3</x:v>
@@ -1490,13 +1486,13 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="22" t="str">
-        <x:v>TEACHING-FOOD-BOX</x:v>
+        <x:v>FURNITURE-OTHER</x:v>
       </x:c>
       <x:c r="B31" s="12" t="str">
-        <x:v>食品真相揭秘箱</x:v>
+        <x:v>其他办公家具及设备</x:v>
       </x:c>
       <x:c r="C31" s="12" t="str">
-        <x:v>TEACHING</x:v>
+        <x:v>FURNITURE</x:v>
       </x:c>
       <x:c r="D31" s="12" t="str">
         <x:v>开启</x:v>
@@ -1505,7 +1501,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="F31" s="12" t="str">
-        <x:v>批量</x:v>
+        <x:v>单件</x:v>
       </x:c>
       <x:c r="G31" s="12" t="str">
         <x:v>件</x:v>
@@ -1522,23 +1518,25 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="22" t="str">
-        <x:v>TEACHING</x:v>
+        <x:v>SUPPLIES-PRINT</x:v>
       </x:c>
       <x:c r="B32" s="12" t="str">
-        <x:v>教学用具</x:v>
-      </x:c>
-      <x:c r="C32" s="12" t="str"/>
+        <x:v>印刷物料</x:v>
+      </x:c>
+      <x:c r="C32" s="12" t="str">
+        <x:v>SUPPLIES</x:v>
+      </x:c>
       <x:c r="D32" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E32" s="12" t="str">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F32" s="12" t="str">
         <x:v>批量</x:v>
       </x:c>
       <x:c r="G32" s="12" t="str">
-        <x:v>件</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="H32" s="12" t="str">
         <x:v>V3</x:v>
@@ -1552,25 +1550,25 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="22" t="str">
-        <x:v>IT-AUDIO-VIDEO</x:v>
+        <x:v>TEACHING-FOOD-BOX</x:v>
       </x:c>
       <x:c r="B33" s="12" t="str">
-        <x:v>音视频设备</x:v>
+        <x:v>食品真相揭秘箱</x:v>
       </x:c>
       <x:c r="C33" s="12" t="str">
-        <x:v>IT</x:v>
+        <x:v>TEACHING</x:v>
       </x:c>
       <x:c r="D33" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E33" s="12" t="str">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F33" s="12" t="str">
-        <x:v>单件</x:v>
+        <x:v>批量</x:v>
       </x:c>
       <x:c r="G33" s="12" t="str">
-        <x:v>台</x:v>
+        <x:v>件</x:v>
       </x:c>
       <x:c r="H33" s="12" t="str">
         <x:v>V3</x:v>
@@ -1584,13 +1582,13 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="22" t="str">
-        <x:v>SUPPLIES-DAILY</x:v>
+        <x:v>IT-AUDIO-VIDEO</x:v>
       </x:c>
       <x:c r="B34" s="12" t="str">
-        <x:v>日杂用品</x:v>
+        <x:v>音视频设备</x:v>
       </x:c>
       <x:c r="C34" s="12" t="str">
-        <x:v>SUPPLIES</x:v>
+        <x:v>IT</x:v>
       </x:c>
       <x:c r="D34" s="12" t="str">
         <x:v>开启</x:v>
@@ -1599,10 +1597,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="F34" s="12" t="str">
-        <x:v>批量</x:v>
+        <x:v>单件</x:v>
       </x:c>
       <x:c r="G34" s="12" t="str">
-        <x:v>个</x:v>
+        <x:v>台</x:v>
       </x:c>
       <x:c r="H34" s="12" t="str">
         <x:v>V3</x:v>
@@ -1616,13 +1614,13 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="22" t="str">
-        <x:v>TEACHING-OTHER</x:v>
+        <x:v>SUPPLIES-DAILY</x:v>
       </x:c>
       <x:c r="B35" s="12" t="str">
-        <x:v>其他教学用具</x:v>
+        <x:v>日杂用品</x:v>
       </x:c>
       <x:c r="C35" s="12" t="str">
-        <x:v>TEACHING</x:v>
+        <x:v>SUPPLIES</x:v>
       </x:c>
       <x:c r="D35" s="12" t="str">
         <x:v>开启</x:v>
@@ -1634,7 +1632,7 @@
         <x:v>批量</x:v>
       </x:c>
       <x:c r="G35" s="12" t="str">
-        <x:v>件</x:v>
+        <x:v>个</x:v>
       </x:c>
       <x:c r="H35" s="12" t="str">
         <x:v>V3</x:v>
@@ -1648,23 +1646,25 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="22" t="str">
-        <x:v>OTHER</x:v>
+        <x:v>TEACHING-OTHER</x:v>
       </x:c>
       <x:c r="B36" s="12" t="str">
-        <x:v>其他</x:v>
-      </x:c>
-      <x:c r="C36" s="12" t="str"/>
+        <x:v>其他教学用具</x:v>
+      </x:c>
+      <x:c r="C36" s="12" t="str">
+        <x:v>TEACHING</x:v>
+      </x:c>
       <x:c r="D36" s="12" t="str">
         <x:v>开启</x:v>
       </x:c>
       <x:c r="E36" s="12" t="str">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F36" s="12" t="str">
-        <x:v>单件</x:v>
+        <x:v>批量</x:v>
       </x:c>
       <x:c r="G36" s="12" t="str">
-        <x:v>个</x:v>
+        <x:v>件</x:v>
       </x:c>
       <x:c r="H36" s="12" t="str">
         <x:v>V3</x:v>

</xml_diff>